<commit_message>
added 2026 rebid xls
</commit_message>
<xml_diff>
--- a/support/2026.xlsx
+++ b/support/2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rcoc-my.sharepoint.com/personal/abates_rcoc_org/Documents/Desktop/Bids/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Purchasing\1 All solicitations in progress\B U-CHANNEL SIGN POSTS\TABS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{3BE1D610-A588-4D2B-AE1A-E4B616017A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{973D0806-E825-414D-A36A-33BEBB1E51BC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{09ED5BA9-48C3-47D2-B0AA-9A4973C1BA38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Price Analysis" sheetId="1" r:id="rId1"/>
@@ -27,9 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="87">
-  <si>
-    <t>Bart Richard Woodward Corporation</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="91">
+  <si>
+    <t>CANUCK POWER INC</t>
+  </si>
+  <si>
+    <t>Decima LLC</t>
   </si>
   <si>
     <t>Dornbos Sign Inc.</t>
@@ -38,22 +41,19 @@
     <t>Eberl Iron Works, Inc.</t>
   </si>
   <si>
-    <t>LINCOLN ALLOY LLC</t>
-  </si>
-  <si>
     <t>Lightle Enterprises of Ohio, LLC</t>
   </si>
   <si>
     <t>MDSolutions</t>
   </si>
   <si>
-    <t>Morgan Ingland LLC</t>
+    <t>Michigan State Industries</t>
   </si>
   <si>
     <t>RATHCO SAFETY SUPPLY</t>
   </si>
   <si>
-    <t>signsverse</t>
+    <t>Vulcan Signs</t>
   </si>
   <si>
     <t>Item No</t>
@@ -109,39 +109,36 @@
     <t>Bid</t>
   </si>
   <si>
+    <t>HEBEI J</t>
+  </si>
+  <si>
+    <t>Nucor</t>
+  </si>
+  <si>
+    <t>1060217</t>
+  </si>
+  <si>
     <t>Franklin Industries</t>
   </si>
   <si>
-    <t>U Channel Post</t>
-  </si>
-  <si>
-    <t>HUC300-120GLV01</t>
-  </si>
-  <si>
-    <t>Nucor</t>
+    <t>HC300-120-12GLV01</t>
   </si>
   <si>
     <t>UC300144HG</t>
   </si>
   <si>
-    <t>LINCOLN ALLOY</t>
-  </si>
-  <si>
-    <t>LAUC123</t>
-  </si>
-  <si>
     <t>3# Galvanized UC</t>
   </si>
   <si>
-    <t>franklin industries</t>
-  </si>
-  <si>
-    <t>2060507</t>
+    <t>MSI</t>
   </si>
   <si>
     <t>12' #3 Galv</t>
   </si>
   <si>
+    <t>3UCGALV-12</t>
+  </si>
+  <si>
     <t>Delivery Address</t>
   </si>
   <si>
@@ -175,20 +172,26 @@
     <t>No</t>
   </si>
   <si>
-    <t>7565 - U-CHANNEL SIGN POSTS, ANNUAL ESTIMATED QUANTITIES</t>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Must be purchased in bundles of 50</t>
   </si>
   <si>
     <t>Road Commission for Oakland County</t>
   </si>
   <si>
-    <t>December 9, 2025 / 2:30 PM</t>
+    <t>April 7, 2026 / 2:30 PM</t>
+  </si>
+  <si>
+    <t>8009 - U-CHANNEL SIGN POSTS, ANNUAL ESTIMATED QUANTITIES, RE-BID</t>
   </si>
   <si>
     <t>TOTALS:</t>
   </si>
   <si>
     <r>
-      <t xml:space="preserve">LINCOLN ALLOY LLC
+      <t xml:space="preserve">MDSolutions
 </t>
     </r>
     <r>
@@ -199,12 +202,12 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>1720 Magnolia Dr
-Yuba City, CA 95991</t>
+      <t>8225 Estates Pkwy
+Plain City, OH 43064</t>
     </r>
   </si>
   <si>
-    <t>Is there an objective or deviation?</t>
+    <t>Is there an objection or deviation?</t>
   </si>
   <si>
     <t>Specify:</t>
@@ -213,16 +216,16 @@
     <t>How long do you anticipate your ability to hold pricing?</t>
   </si>
   <si>
-    <t>360 days</t>
-  </si>
-  <si>
-    <t>Minimum order requirements.</t>
+    <t>1 year</t>
+  </si>
+  <si>
+    <t>Minimum order requirements:</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
   <si>
     <t>Indicate number of days for delivery to RCOC after receipt of order:</t>
-  </si>
-  <si>
-    <t>14 days after initial 60 days production period</t>
   </si>
   <si>
     <t>Indicate how many item rolls are packaged in standard bundle:</t>
@@ -247,29 +250,6 @@
   </si>
   <si>
     <t>Bid Solicitation Doc(s) Returned / Uploaded</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Dornbos Sign Inc.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>619 W. Harris St.
-Charlotte, MI 48813</t>
-    </r>
-  </si>
-  <si>
-    <t>N/A</t>
   </si>
   <si>
     <r>
@@ -289,73 +269,10 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">1 year </t>
-  </si>
-  <si>
-    <t>20,000 LBs</t>
-  </si>
-  <si>
-    <t>60 days</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">MDSolutions
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>8225 Estates Pkwy
-Plain City, OH 43064</t>
-    </r>
-  </si>
-  <si>
-    <t>1 year</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">signsverse
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>5822 Providence Oak
-San Antonio, TX 78249</t>
-    </r>
-  </si>
-  <si>
-    <t>90 days</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Morgan Ingland LLC
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>380 Tennant Ave. Unit 3
-Morgan Hill, CA 95037</t>
-    </r>
-  </si>
-  <si>
-    <t>4-5 weeks</t>
+    <t>20,000 lbs</t>
+  </si>
+  <si>
+    <t>45-60 days</t>
   </si>
   <si>
     <r>
@@ -379,6 +296,101 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">CANUCK POWER INC
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>1720 Magnolia Dr
+Yuba City, CA 95991</t>
+    </r>
+  </si>
+  <si>
+    <t>360 days</t>
+  </si>
+  <si>
+    <t>90 for first order, 7 days after</t>
+  </si>
+  <si>
+    <t>50 to 100</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Michigan State Industries
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>206 E. Michigan Ave P.O. Box 30723
+Lansing, MI 48909</t>
+    </r>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>30 days</t>
+  </si>
+  <si>
+    <t>1,000 posts</t>
+  </si>
+  <si>
+    <t>50 per bundle</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dornbos Sign Inc.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>6619 W. Harris St.
+Charlotte, MI 48813</t>
+    </r>
+  </si>
+  <si>
+    <t>60 days</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Vulcan Signs
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>P.O. Box 1850
+Foley, AL 36536</t>
+    </r>
+  </si>
+  <si>
+    <t>30-45 days</t>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">Lightle Enterprises of Ohio, LLC
 </t>
     </r>
@@ -395,17 +407,17 @@
     </r>
   </si>
   <si>
-    <t>One year</t>
-  </si>
-  <si>
-    <t>1000 EA. Post</t>
-  </si>
-  <si>
-    <t>30-90</t>
+    <t>6 months</t>
+  </si>
+  <si>
+    <t>45-90</t>
+  </si>
+  <si>
+    <t>U-channel post 50 bundle, square post 25/bundle</t>
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Bart Richard Woodward Corporation
+      <t xml:space="preserve">Decima LLC
 </t>
     </r>
     <r>
@@ -416,30 +428,29 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>601 E Main Street
-Medaryville, IN 47957</t>
+      <t>16870 Schaefer Hwy
+Detroit, MI 48235</t>
     </r>
   </si>
   <si>
-    <t>12 months</t>
-  </si>
-  <si>
-    <t>50-piece bundles</t>
-  </si>
-  <si>
-    <t>Item Number</t>
+    <t>1 month</t>
+  </si>
+  <si>
+    <t>Minimum order is 1,000 units</t>
+  </si>
+  <si>
+    <t>14-18 weeks</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -519,13 +530,6 @@
       <i/>
       <sz val="11"/>
       <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -592,15 +596,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -651,6 +646,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -697,40 +701,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -742,29 +748,31 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="6" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1099,79 +1107,75 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.28515625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13" style="4" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" style="4" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" style="4" customWidth="1"/>
-    <col min="10" max="10" width="10" style="4" customWidth="1"/>
-    <col min="11" max="11" width="13.5703125" style="4" customWidth="1"/>
-    <col min="12" max="12" width="15" style="4" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.85546875" style="4" customWidth="1"/>
-    <col min="15" max="15" width="13.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="36.5703125" style="4" customWidth="1"/>
-    <col min="17" max="17" width="12" style="4" customWidth="1"/>
-    <col min="18" max="18" width="12.7109375" style="4" customWidth="1"/>
-    <col min="19" max="19" width="14" style="4" customWidth="1"/>
-    <col min="20" max="20" width="13.28515625" style="4" customWidth="1"/>
-    <col min="21" max="21" width="9.85546875" style="4" customWidth="1"/>
-    <col min="22" max="22" width="13" style="4" customWidth="1"/>
-    <col min="23" max="23" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="17.7109375" style="4" customWidth="1"/>
-    <col min="25" max="25" width="10.28515625" style="4" customWidth="1"/>
-    <col min="26" max="26" width="12.28515625" style="4" customWidth="1"/>
-    <col min="27" max="27" width="12.7109375" style="4" customWidth="1"/>
-    <col min="28" max="28" width="15.28515625" style="4" customWidth="1"/>
-    <col min="29" max="29" width="11.85546875" style="4" customWidth="1"/>
-    <col min="30" max="30" width="12.28515625" style="4" customWidth="1"/>
-    <col min="31" max="31" width="12.7109375" style="4" customWidth="1"/>
-    <col min="32" max="32" width="15.28515625" style="4" customWidth="1"/>
-    <col min="33" max="33" width="11.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.28515625" style="4" customWidth="1"/>
-    <col min="36" max="36" width="14.5703125" style="4" customWidth="1"/>
-    <col min="37" max="37" width="10.85546875" style="4" customWidth="1"/>
-    <col min="38" max="38" width="8.7109375" style="4" customWidth="1"/>
-    <col min="39" max="39" width="14" style="4" customWidth="1"/>
-    <col min="40" max="40" width="15" style="4" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="10.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="6.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="11.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="10.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="46" max="47" width="50" style="4" customWidth="1"/>
-    <col min="48" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="33" style="5" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" style="5" customWidth="1"/>
+    <col min="9" max="9" width="12" style="5" customWidth="1"/>
+    <col min="10" max="10" width="11.140625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="12.85546875" style="5" customWidth="1"/>
+    <col min="12" max="12" width="15" style="5" customWidth="1"/>
+    <col min="13" max="13" width="9.5703125" style="5" customWidth="1"/>
+    <col min="14" max="14" width="10.85546875" style="5" customWidth="1"/>
+    <col min="15" max="15" width="14.28515625" style="5" customWidth="1"/>
+    <col min="16" max="16" width="14" style="5" customWidth="1"/>
+    <col min="17" max="17" width="9.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" style="5" customWidth="1"/>
+    <col min="19" max="19" width="13.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.28515625" style="5" customWidth="1"/>
+    <col min="21" max="21" width="9.140625" style="5"/>
+    <col min="22" max="22" width="10.85546875" style="5" customWidth="1"/>
+    <col min="23" max="23" width="14.7109375" style="5" customWidth="1"/>
+    <col min="24" max="24" width="16.140625" style="5" customWidth="1"/>
+    <col min="25" max="25" width="11.42578125" style="5" customWidth="1"/>
+    <col min="26" max="26" width="11.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.140625" style="5" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" style="5" customWidth="1"/>
+    <col min="30" max="30" width="11.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.140625" style="5" customWidth="1"/>
+    <col min="32" max="32" width="16" style="5" customWidth="1"/>
+    <col min="33" max="33" width="13.140625" style="5" customWidth="1"/>
+    <col min="34" max="34" width="11" style="5" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" style="5" customWidth="1"/>
+    <col min="36" max="36" width="14.85546875" style="5" customWidth="1"/>
+    <col min="37" max="37" width="10.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.140625" style="5" customWidth="1"/>
+    <col min="39" max="39" width="13" style="5" customWidth="1"/>
+    <col min="40" max="40" width="12.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="10.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="6.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="11.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="45" max="46" width="50" style="5" customWidth="1"/>
+    <col min="47" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
-        <v>48</v>
+      <c r="A2" s="6" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="51.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
+    <row r="5" spans="1:15" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D5" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
@@ -1183,7 +1187,7 @@
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
       <c r="L5" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M5" s="14"/>
       <c r="N5" s="14"/>
@@ -1191,24 +1195,24 @@
     </row>
     <row r="6" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B6" s="15"/>
       <c r="C6" s="16"/>
       <c r="D6" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E6" s="20"/>
       <c r="F6" s="20"/>
       <c r="G6" s="21"/>
       <c r="H6" s="19" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="I6" s="20"/>
       <c r="J6" s="20"/>
       <c r="K6" s="21"/>
       <c r="L6" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M6" s="20"/>
       <c r="N6" s="20"/>
@@ -1216,7 +1220,7 @@
     </row>
     <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="16"/>
@@ -1235,22 +1239,24 @@
     </row>
     <row r="8" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="16"/>
       <c r="D8" s="19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E8" s="20"/>
       <c r="F8" s="20"/>
       <c r="G8" s="21"/>
-      <c r="H8" s="19"/>
+      <c r="H8" s="19" t="s">
+        <v>57</v>
+      </c>
       <c r="I8" s="20"/>
       <c r="J8" s="20"/>
       <c r="K8" s="21"/>
       <c r="L8" s="19" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="M8" s="20"/>
       <c r="N8" s="20"/>
@@ -1258,22 +1264,24 @@
     </row>
     <row r="9" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="16"/>
-      <c r="D9" s="27">
-        <v>10000</v>
+      <c r="D9" s="19" t="s">
+        <v>59</v>
       </c>
       <c r="E9" s="20"/>
       <c r="F9" s="20"/>
       <c r="G9" s="21"/>
-      <c r="H9" s="19"/>
+      <c r="H9" s="19" t="s">
+        <v>66</v>
+      </c>
       <c r="I9" s="20"/>
       <c r="J9" s="20"/>
       <c r="K9" s="21"/>
-      <c r="L9" s="19" t="s">
-        <v>69</v>
+      <c r="L9" s="19">
+        <v>500</v>
       </c>
       <c r="M9" s="20"/>
       <c r="N9" s="20"/>
@@ -1281,22 +1289,24 @@
     </row>
     <row r="10" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="16"/>
-      <c r="D10" s="19" t="s">
-        <v>59</v>
+      <c r="D10" s="19">
+        <v>45</v>
       </c>
       <c r="E10" s="20"/>
       <c r="F10" s="20"/>
       <c r="G10" s="21"/>
-      <c r="H10" s="19"/>
+      <c r="H10" s="19" t="s">
+        <v>67</v>
+      </c>
       <c r="I10" s="20"/>
       <c r="J10" s="20"/>
       <c r="K10" s="21"/>
-      <c r="L10" s="19" t="s">
-        <v>70</v>
+      <c r="L10" s="19">
+        <v>120</v>
       </c>
       <c r="M10" s="20"/>
       <c r="N10" s="20"/>
@@ -1304,17 +1314,19 @@
     </row>
     <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="16"/>
       <c r="D11" s="19">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E11" s="20"/>
       <c r="F11" s="20"/>
       <c r="G11" s="21"/>
-      <c r="H11" s="19"/>
+      <c r="H11" s="19">
+        <v>50</v>
+      </c>
       <c r="I11" s="20"/>
       <c r="J11" s="20"/>
       <c r="K11" s="21"/>
@@ -1327,17 +1339,19 @@
     </row>
     <row r="12" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="16"/>
       <c r="D12" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E12" s="20"/>
       <c r="F12" s="20"/>
       <c r="G12" s="21"/>
-      <c r="H12" s="19"/>
+      <c r="H12" s="19" t="s">
+        <v>46</v>
+      </c>
       <c r="I12" s="20"/>
       <c r="J12" s="20"/>
       <c r="K12" s="21"/>
@@ -1350,7 +1364,7 @@
     </row>
     <row r="13" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="16"/>
@@ -1362,19 +1376,21 @@
       <c r="I13" s="20"/>
       <c r="J13" s="20"/>
       <c r="K13" s="21"/>
-      <c r="L13" s="19"/>
+      <c r="L13" s="19" t="s">
+        <v>69</v>
+      </c>
       <c r="M13" s="20"/>
       <c r="N13" s="20"/>
       <c r="O13" s="21"/>
     </row>
     <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="25"/>
       <c r="C14" s="26"/>
       <c r="D14" s="19" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="E14" s="20"/>
       <c r="F14" s="20"/>
@@ -1386,7 +1402,7 @@
       <c r="J14" s="20"/>
       <c r="K14" s="21"/>
       <c r="L14" s="19" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="M14" s="20"/>
       <c r="N14" s="20"/>
@@ -1439,7 +1455,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>22</v>
       </c>
@@ -1449,83 +1465,80 @@
       <c r="C16" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="11">
+        <v>36.15</v>
+      </c>
+      <c r="G16" s="11">
+        <v>108450</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="J16" s="11">
+        <v>36.950000000000003</v>
+      </c>
+      <c r="K16" s="11">
+        <v>110850</v>
+      </c>
+      <c r="L16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="M16" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F16" s="10">
-        <v>35</v>
-      </c>
-      <c r="G16" s="10">
-        <v>105000</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="J16" s="10">
-        <v>36.36</v>
-      </c>
-      <c r="K16" s="10">
-        <v>109080</v>
-      </c>
-      <c r="L16" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="M16" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="N16" s="10">
-        <v>37</v>
-      </c>
-      <c r="O16" s="10">
-        <v>111000</v>
+      <c r="N16" s="11">
+        <v>39.74</v>
+      </c>
+      <c r="O16" s="11">
+        <v>119220</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="22" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="24"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
       <c r="F17" s="17">
-        <v>105000</v>
+        <v>108450</v>
       </c>
       <c r="G17" s="18"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
       <c r="J17" s="17">
-        <v>109080</v>
+        <v>110850</v>
       </c>
       <c r="K17" s="18"/>
       <c r="L17" s="12"/>
       <c r="M17" s="12"/>
       <c r="N17" s="17">
-        <v>111000</v>
+        <v>119220</v>
       </c>
       <c r="O17" s="18"/>
     </row>
-    <row r="19" spans="1:15" ht="51.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:15" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D19" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E19" s="14"/>
       <c r="F19" s="14"/>
       <c r="G19" s="14"/>
       <c r="H19" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I19" s="14"/>
       <c r="J19" s="14"/>
       <c r="K19" s="14"/>
       <c r="L19" s="13" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="M19" s="14"/>
       <c r="N19" s="14"/>
@@ -1533,24 +1546,24 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B20" s="15"/>
       <c r="C20" s="16"/>
       <c r="D20" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E20" s="20"/>
       <c r="F20" s="20"/>
       <c r="G20" s="21"/>
       <c r="H20" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I20" s="20"/>
       <c r="J20" s="20"/>
       <c r="K20" s="21"/>
       <c r="L20" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M20" s="20"/>
       <c r="N20" s="20"/>
@@ -1558,7 +1571,7 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B21" s="15"/>
       <c r="C21" s="16"/>
@@ -1566,7 +1579,9 @@
       <c r="E21" s="20"/>
       <c r="F21" s="20"/>
       <c r="G21" s="21"/>
-      <c r="H21" s="19"/>
+      <c r="H21" s="19" t="s">
+        <v>75</v>
+      </c>
       <c r="I21" s="20"/>
       <c r="J21" s="20"/>
       <c r="K21" s="21"/>
@@ -1577,24 +1592,24 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="16"/>
       <c r="D22" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E22" s="20"/>
       <c r="F22" s="20"/>
       <c r="G22" s="21"/>
       <c r="H22" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I22" s="20"/>
       <c r="J22" s="20"/>
       <c r="K22" s="21"/>
       <c r="L22" s="19" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="M22" s="20"/>
       <c r="N22" s="20"/>
@@ -1602,22 +1617,24 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="16"/>
-      <c r="D23" s="19"/>
+      <c r="D23" s="27">
+        <v>30000</v>
+      </c>
       <c r="E23" s="20"/>
       <c r="F23" s="20"/>
       <c r="G23" s="21"/>
-      <c r="H23" s="19">
-        <v>500</v>
+      <c r="H23" s="19" t="s">
+        <v>77</v>
       </c>
       <c r="I23" s="20"/>
       <c r="J23" s="20"/>
       <c r="K23" s="21"/>
       <c r="L23" s="19" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="M23" s="20"/>
       <c r="N23" s="20"/>
@@ -1625,24 +1642,24 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="16"/>
-      <c r="D24" s="19">
-        <v>45</v>
+      <c r="D24" s="19" t="s">
+        <v>72</v>
       </c>
       <c r="E24" s="20"/>
       <c r="F24" s="20"/>
       <c r="G24" s="21"/>
-      <c r="H24" s="19">
-        <v>45</v>
+      <c r="H24" s="19" t="s">
+        <v>76</v>
       </c>
       <c r="I24" s="20"/>
       <c r="J24" s="20"/>
       <c r="K24" s="21"/>
       <c r="L24" s="19" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="M24" s="20"/>
       <c r="N24" s="20"/>
@@ -1650,55 +1667,55 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="16"/>
-      <c r="D25" s="19">
-        <v>50</v>
+      <c r="D25" s="19" t="s">
+        <v>73</v>
       </c>
       <c r="E25" s="20"/>
       <c r="F25" s="20"/>
       <c r="G25" s="21"/>
-      <c r="H25" s="19">
-        <v>25</v>
+      <c r="H25" s="19" t="s">
+        <v>78</v>
       </c>
       <c r="I25" s="20"/>
       <c r="J25" s="20"/>
       <c r="K25" s="21"/>
-      <c r="L25" s="19"/>
+      <c r="L25" s="19" t="s">
+        <v>78</v>
+      </c>
       <c r="M25" s="20"/>
       <c r="N25" s="20"/>
       <c r="O25" s="21"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="16"/>
       <c r="D26" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E26" s="20"/>
       <c r="F26" s="20"/>
       <c r="G26" s="21"/>
       <c r="H26" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I26" s="20"/>
       <c r="J26" s="20"/>
       <c r="K26" s="21"/>
-      <c r="L26" s="19" t="s">
-        <v>47</v>
-      </c>
+      <c r="L26" s="19"/>
       <c r="M26" s="20"/>
       <c r="N26" s="20"/>
       <c r="O26" s="21"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B27" s="15"/>
       <c r="C27" s="16"/>
@@ -1706,7 +1723,9 @@
       <c r="E27" s="20"/>
       <c r="F27" s="20"/>
       <c r="G27" s="21"/>
-      <c r="H27" s="19"/>
+      <c r="H27" s="19" t="s">
+        <v>75</v>
+      </c>
       <c r="I27" s="20"/>
       <c r="J27" s="20"/>
       <c r="K27" s="21"/>
@@ -1717,24 +1736,24 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B28" s="25"/>
       <c r="C28" s="26"/>
       <c r="D28" s="19" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="E28" s="20"/>
       <c r="F28" s="20"/>
       <c r="G28" s="21"/>
       <c r="H28" s="19" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="I28" s="20"/>
       <c r="J28" s="20"/>
       <c r="K28" s="21"/>
       <c r="L28" s="19" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="M28" s="20"/>
       <c r="N28" s="20"/>
@@ -1797,104 +1816,83 @@
       <c r="C30" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="10">
-        <v>37.119999999999997</v>
-      </c>
-      <c r="G30" s="10">
-        <v>111360</v>
-      </c>
-      <c r="H30" s="11"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="10">
-        <v>38</v>
-      </c>
-      <c r="K30" s="10">
-        <v>114000</v>
+      <c r="D30" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="10"/>
+      <c r="F30" s="11">
+        <v>40</v>
+      </c>
+      <c r="G30" s="11">
+        <v>120000</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I30" s="10"/>
+      <c r="J30" s="11">
+        <v>40</v>
+      </c>
+      <c r="K30" s="11">
+        <v>120000</v>
       </c>
       <c r="L30" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="M30" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="N30" s="10">
-        <v>40.29</v>
-      </c>
-      <c r="O30" s="10">
-        <v>120870</v>
+        <v>29</v>
+      </c>
+      <c r="M30" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="N30" s="11">
+        <v>40.049999999999997</v>
+      </c>
+      <c r="O30" s="11">
+        <v>120150</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A31" s="22" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B31" s="23"/>
       <c r="C31" s="24"/>
       <c r="D31" s="12"/>
       <c r="E31" s="12"/>
       <c r="F31" s="17">
-        <v>111360</v>
+        <v>120000</v>
       </c>
       <c r="G31" s="18"/>
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
       <c r="J31" s="17">
-        <v>114000</v>
+        <v>120000</v>
       </c>
       <c r="K31" s="18"/>
       <c r="L31" s="12"/>
       <c r="M31" s="12"/>
       <c r="N31" s="17">
-        <v>120870</v>
+        <v>120150</v>
       </c>
       <c r="O31" s="18"/>
     </row>
-    <row r="38" spans="1:15" ht="51.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D38" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="I38" s="14"/>
-      <c r="J38" s="14"/>
-      <c r="K38" s="14"/>
-      <c r="L38" s="13" t="s">
+    <row r="39" spans="1:15" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D39" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="M38" s="14"/>
-      <c r="N38" s="14"/>
-      <c r="O38" s="14"/>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A39" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="B39" s="15"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="E39" s="20"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="21"/>
-      <c r="H39" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="I39" s="20"/>
-      <c r="J39" s="20"/>
-      <c r="K39" s="21"/>
-      <c r="L39" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="M39" s="20"/>
-      <c r="N39" s="20"/>
-      <c r="O39" s="21"/>
+      <c r="I39" s="14"/>
+      <c r="J39" s="14"/>
+      <c r="K39" s="14"/>
+      <c r="L39" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="M39" s="14"/>
+      <c r="N39" s="14"/>
+      <c r="O39" s="14"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
@@ -1903,16 +1901,20 @@
       <c r="B40" s="15"/>
       <c r="C40" s="16"/>
       <c r="D40" s="19" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="E40" s="20"/>
       <c r="F40" s="20"/>
       <c r="G40" s="21"/>
-      <c r="H40" s="19"/>
+      <c r="H40" s="19" t="s">
+        <v>46</v>
+      </c>
       <c r="I40" s="20"/>
       <c r="J40" s="20"/>
       <c r="K40" s="21"/>
-      <c r="L40" s="19"/>
+      <c r="L40" s="19" t="s">
+        <v>46</v>
+      </c>
       <c r="M40" s="20"/>
       <c r="N40" s="20"/>
       <c r="O40" s="21"/>
@@ -1923,45 +1925,39 @@
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="16"/>
-      <c r="D41" s="19" t="s">
-        <v>72</v>
-      </c>
+      <c r="D41" s="19"/>
       <c r="E41" s="20"/>
       <c r="F41" s="20"/>
       <c r="G41" s="21"/>
-      <c r="H41" s="19" t="s">
-        <v>80</v>
-      </c>
+      <c r="H41" s="19"/>
       <c r="I41" s="20"/>
       <c r="J41" s="20"/>
       <c r="K41" s="21"/>
-      <c r="L41" s="19" t="s">
-        <v>84</v>
-      </c>
+      <c r="L41" s="19"/>
       <c r="M41" s="20"/>
       <c r="N41" s="20"/>
       <c r="O41" s="21"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B42" s="15"/>
       <c r="C42" s="16"/>
-      <c r="D42" s="27">
-        <v>500</v>
+      <c r="D42" s="28">
+        <v>46387</v>
       </c>
       <c r="E42" s="20"/>
       <c r="F42" s="20"/>
       <c r="G42" s="21"/>
       <c r="H42" s="19" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="I42" s="20"/>
       <c r="J42" s="20"/>
       <c r="K42" s="21"/>
       <c r="L42" s="19" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="M42" s="20"/>
       <c r="N42" s="20"/>
@@ -1973,20 +1969,18 @@
       </c>
       <c r="B43" s="15"/>
       <c r="C43" s="16"/>
-      <c r="D43" s="19">
-        <v>45</v>
+      <c r="D43" s="19" t="s">
+        <v>48</v>
       </c>
       <c r="E43" s="20"/>
       <c r="F43" s="20"/>
       <c r="G43" s="21"/>
-      <c r="H43" s="19" t="s">
-        <v>82</v>
-      </c>
+      <c r="H43" s="19"/>
       <c r="I43" s="20"/>
       <c r="J43" s="20"/>
       <c r="K43" s="21"/>
       <c r="L43" s="19" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="M43" s="20"/>
       <c r="N43" s="20"/>
@@ -1998,20 +1992,20 @@
       </c>
       <c r="B44" s="15"/>
       <c r="C44" s="16"/>
-      <c r="D44" s="19">
-        <v>50</v>
+      <c r="D44" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="E44" s="20"/>
       <c r="F44" s="20"/>
       <c r="G44" s="21"/>
-      <c r="H44" s="19">
-        <v>50</v>
+      <c r="H44" s="19" t="s">
+        <v>85</v>
       </c>
       <c r="I44" s="20"/>
       <c r="J44" s="20"/>
       <c r="K44" s="21"/>
-      <c r="L44" s="19">
-        <v>50</v>
+      <c r="L44" s="19" t="s">
+        <v>90</v>
       </c>
       <c r="M44" s="20"/>
       <c r="N44" s="20"/>
@@ -2023,21 +2017,19 @@
       </c>
       <c r="B45" s="15"/>
       <c r="C45" s="16"/>
-      <c r="D45" s="19" t="s">
-        <v>64</v>
+      <c r="D45" s="19">
+        <v>50</v>
       </c>
       <c r="E45" s="20"/>
       <c r="F45" s="20"/>
       <c r="G45" s="21"/>
       <c r="H45" s="19" t="s">
-        <v>47</v>
+        <v>86</v>
       </c>
       <c r="I45" s="20"/>
       <c r="J45" s="20"/>
       <c r="K45" s="21"/>
-      <c r="L45" s="19" t="s">
-        <v>47</v>
-      </c>
+      <c r="L45" s="19"/>
       <c r="M45" s="20"/>
       <c r="N45" s="20"/>
       <c r="O45" s="21"/>
@@ -2049,179 +2041,204 @@
       <c r="B46" s="15"/>
       <c r="C46" s="16"/>
       <c r="D46" s="19" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="E46" s="20"/>
       <c r="F46" s="20"/>
       <c r="G46" s="21"/>
-      <c r="H46" s="19"/>
+      <c r="H46" s="19" t="s">
+        <v>46</v>
+      </c>
       <c r="I46" s="20"/>
       <c r="J46" s="20"/>
       <c r="K46" s="21"/>
-      <c r="L46" s="19"/>
+      <c r="L46" s="19" t="s">
+        <v>46</v>
+      </c>
       <c r="M46" s="20"/>
       <c r="N46" s="20"/>
       <c r="O46" s="21"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A47" s="25" t="s">
+      <c r="A47" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="B47" s="25"/>
-      <c r="C47" s="26"/>
-      <c r="D47" s="19" t="s">
-        <v>64</v>
-      </c>
+      <c r="B47" s="15"/>
+      <c r="C47" s="16"/>
+      <c r="D47" s="19"/>
       <c r="E47" s="20"/>
       <c r="F47" s="20"/>
       <c r="G47" s="21"/>
-      <c r="H47" s="19" t="s">
-        <v>64</v>
-      </c>
+      <c r="H47" s="19"/>
       <c r="I47" s="20"/>
       <c r="J47" s="20"/>
       <c r="K47" s="21"/>
-      <c r="L47" s="19" t="s">
-        <v>64</v>
-      </c>
+      <c r="L47" s="19"/>
       <c r="M47" s="20"/>
       <c r="N47" s="20"/>
       <c r="O47" s="21"/>
     </row>
-    <row r="48" spans="1:15" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="7" t="s">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A48" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B48" s="25"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="E48" s="20"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="21"/>
+      <c r="H48" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="I48" s="20"/>
+      <c r="J48" s="20"/>
+      <c r="K48" s="21"/>
+      <c r="L48" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="M48" s="20"/>
+      <c r="N48" s="20"/>
+      <c r="O48" s="21"/>
+    </row>
+    <row r="49" spans="1:15" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B48" s="7" t="s">
+      <c r="B49" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="C49" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D48" s="7" t="s">
+      <c r="D49" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E48" s="7" t="s">
+      <c r="E49" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F48" s="7" t="s">
+      <c r="F49" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="G48" s="7" t="s">
+      <c r="G49" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H48" s="7" t="s">
+      <c r="H49" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="I48" s="7" t="s">
+      <c r="I49" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="J48" s="7" t="s">
+      <c r="J49" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="K48" s="7" t="s">
+      <c r="K49" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="L48" s="7" t="s">
+      <c r="L49" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M48" s="7" t="s">
+      <c r="M49" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N48" s="7" t="s">
+      <c r="N49" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="O48" s="7" t="s">
+      <c r="O49" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="49" spans="1:15" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="8" t="s">
+    <row r="50" spans="1:15" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B49" s="9">
+      <c r="B50" s="9">
         <v>3000</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C50" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D49" s="11" t="s">
+      <c r="D50" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F50" s="11">
+        <v>42.84</v>
+      </c>
+      <c r="G50" s="11">
+        <v>128520</v>
+      </c>
+      <c r="H50" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E49" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="F49" s="10">
-        <v>40.5</v>
-      </c>
-      <c r="G49" s="10">
-        <v>121500</v>
-      </c>
-      <c r="H49" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I49" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J49" s="10">
-        <v>44.88</v>
-      </c>
-      <c r="K49" s="10">
-        <v>134640</v>
-      </c>
-      <c r="L49" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="M49" s="8" t="s">
+      <c r="I50" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="J50" s="11">
+        <v>47.6</v>
+      </c>
+      <c r="K50" s="11">
+        <v>142800</v>
+      </c>
+      <c r="L50" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="N49" s="10">
-        <v>69.5</v>
-      </c>
-      <c r="O49" s="10">
-        <v>208500</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B50" s="23"/>
-      <c r="C50" s="24"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="12"/>
-      <c r="F50" s="17">
-        <v>121500</v>
-      </c>
-      <c r="G50" s="18"/>
-      <c r="H50" s="12"/>
-      <c r="I50" s="12"/>
-      <c r="J50" s="17">
-        <v>134640</v>
-      </c>
-      <c r="K50" s="18"/>
-      <c r="L50" s="12"/>
-      <c r="M50" s="12"/>
-      <c r="N50" s="17">
-        <v>208500</v>
-      </c>
-      <c r="O50" s="18"/>
+      <c r="M50" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N50" s="11">
+        <v>56</v>
+      </c>
+      <c r="O50" s="11">
+        <v>168000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51" s="23"/>
+      <c r="C51" s="24"/>
+      <c r="D51" s="12"/>
+      <c r="E51" s="12"/>
+      <c r="F51" s="17">
+        <v>128520</v>
+      </c>
+      <c r="G51" s="18"/>
+      <c r="H51" s="12"/>
+      <c r="I51" s="12"/>
+      <c r="J51" s="17">
+        <v>142800</v>
+      </c>
+      <c r="K51" s="18"/>
+      <c r="L51" s="12"/>
+      <c r="M51" s="12"/>
+      <c r="N51" s="17">
+        <v>168000</v>
+      </c>
+      <c r="O51" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="129">
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A46:C46"/>
     <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A42:C42"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A22:C22"/>
@@ -2231,29 +2248,36 @@
     <mergeCell ref="D13:G13"/>
     <mergeCell ref="H13:K13"/>
     <mergeCell ref="L13:O13"/>
-    <mergeCell ref="L39:O39"/>
+    <mergeCell ref="D27:G27"/>
     <mergeCell ref="L40:O40"/>
     <mergeCell ref="L41:O41"/>
     <mergeCell ref="L42:O42"/>
     <mergeCell ref="L43:O43"/>
-    <mergeCell ref="D44:G44"/>
-    <mergeCell ref="D45:G45"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="H26:K26"/>
+    <mergeCell ref="H28:K28"/>
+    <mergeCell ref="L20:O20"/>
+    <mergeCell ref="L21:O21"/>
+    <mergeCell ref="L22:O22"/>
+    <mergeCell ref="L23:O23"/>
+    <mergeCell ref="L24:O24"/>
+    <mergeCell ref="L25:O25"/>
+    <mergeCell ref="L26:O26"/>
+    <mergeCell ref="L28:O28"/>
+    <mergeCell ref="H27:K27"/>
+    <mergeCell ref="L27:O27"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="H45:K45"/>
+    <mergeCell ref="H46:K46"/>
+    <mergeCell ref="H48:K48"/>
     <mergeCell ref="D47:G47"/>
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="H40:K40"/>
-    <mergeCell ref="H41:K41"/>
-    <mergeCell ref="H42:K42"/>
-    <mergeCell ref="H43:K43"/>
-    <mergeCell ref="H44:K44"/>
-    <mergeCell ref="H45:K45"/>
     <mergeCell ref="H47:K47"/>
-    <mergeCell ref="D46:G46"/>
-    <mergeCell ref="H46:K46"/>
-    <mergeCell ref="D39:G39"/>
     <mergeCell ref="D40:G40"/>
     <mergeCell ref="D41:G41"/>
     <mergeCell ref="D42:G42"/>
     <mergeCell ref="D43:G43"/>
+    <mergeCell ref="D44:G44"/>
     <mergeCell ref="L11:O11"/>
     <mergeCell ref="L12:O12"/>
     <mergeCell ref="L14:O14"/>
@@ -2262,21 +2286,12 @@
     <mergeCell ref="D22:G22"/>
     <mergeCell ref="D23:G23"/>
     <mergeCell ref="D24:G24"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="H25:K25"/>
-    <mergeCell ref="L20:O20"/>
-    <mergeCell ref="L21:O21"/>
-    <mergeCell ref="L22:O22"/>
-    <mergeCell ref="L23:O23"/>
-    <mergeCell ref="L24:O24"/>
-    <mergeCell ref="L25:O25"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="L44:O44"/>
+    <mergeCell ref="H40:K40"/>
+    <mergeCell ref="H41:K41"/>
+    <mergeCell ref="H42:K42"/>
+    <mergeCell ref="H43:K43"/>
+    <mergeCell ref="H44:K44"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="H7:K7"/>
     <mergeCell ref="H8:K8"/>
@@ -2290,39 +2305,37 @@
     <mergeCell ref="D8:G8"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="D10:G10"/>
-    <mergeCell ref="J50:K50"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="L44:O44"/>
+    <mergeCell ref="J51:K51"/>
+    <mergeCell ref="N51:O51"/>
     <mergeCell ref="L45:O45"/>
+    <mergeCell ref="L46:O46"/>
+    <mergeCell ref="L48:O48"/>
     <mergeCell ref="L47:O47"/>
-    <mergeCell ref="L46:O46"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="J17:K17"/>
     <mergeCell ref="N17:O17"/>
     <mergeCell ref="F31:G31"/>
     <mergeCell ref="J31:K31"/>
     <mergeCell ref="N31:O31"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="L38:O38"/>
-    <mergeCell ref="H38:K38"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="L39:O39"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="D25:G25"/>
     <mergeCell ref="D26:G26"/>
     <mergeCell ref="D28:G28"/>
-    <mergeCell ref="H26:K26"/>
-    <mergeCell ref="H28:K28"/>
-    <mergeCell ref="L26:O26"/>
-    <mergeCell ref="L28:O28"/>
-    <mergeCell ref="H27:K27"/>
-    <mergeCell ref="L27:O27"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="D38:G38"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="D45:G45"/>
+    <mergeCell ref="D46:G46"/>
+    <mergeCell ref="D48:G48"/>
+    <mergeCell ref="D39:G39"/>
     <mergeCell ref="L19:O19"/>
     <mergeCell ref="H19:K19"/>
     <mergeCell ref="D19:G19"/>
     <mergeCell ref="L5:O5"/>
     <mergeCell ref="H5:K5"/>
     <mergeCell ref="D5:G5"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A40:C40"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A8:C8"/>
@@ -2338,47 +2351,44 @@
     <mergeCell ref="L9:O9"/>
     <mergeCell ref="L10:O10"/>
     <mergeCell ref="D11:G11"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="D14:G14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="3" scale="90" orientation="landscape" r:id="rId1"/>
-  <headerFooter>
-    <oddFooter>&amp;R&amp;8&amp;F
-Page &amp;P of &amp;N</oddFooter>
-  </headerFooter>
+  <pageSetup paperSize="3" scale="90" fitToWidth="0" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
-        <v>86</v>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>37</v>
@@ -2393,32 +2403,26 @@
         <v>40</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="L1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
         <v>23</v>
       </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
       <c r="J2" t="s">
-        <v>22</v>
-      </c>
-      <c r="K2" t="s">
         <v>24</v>
       </c>
-      <c r="L2">
+      <c r="K2">
         <v>3000</v>
       </c>
     </row>
@@ -2433,9 +2437,9 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6.28515625" bestFit="1" customWidth="1"/>
@@ -2449,7 +2453,7 @@
         <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
@@ -2489,23 +2493,20 @@
       <c r="C2" t="s">
         <v>26</v>
       </c>
-      <c r="D2" t="s">
-        <v>27</v>
-      </c>
       <c r="E2" t="s">
         <v>25</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G2">
         <v>3000</v>
       </c>
       <c r="H2">
-        <v>69.5</v>
+        <v>40</v>
       </c>
       <c r="I2">
-        <v>208500</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -2516,7 +2517,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
         <v>28</v>
@@ -2525,16 +2526,16 @@
         <v>25</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G3">
         <v>3000</v>
       </c>
       <c r="H3">
-        <v>36.36</v>
+        <v>56</v>
       </c>
       <c r="I3">
-        <v>109080</v>
+        <v>168000</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -2554,16 +2555,16 @@
         <v>25</v>
       </c>
       <c r="F4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G4">
         <v>3000</v>
       </c>
       <c r="H4">
-        <v>40.5</v>
+        <v>40.049999999999997</v>
       </c>
       <c r="I4">
-        <v>121500</v>
+        <v>120150</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -2574,25 +2575,25 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
         <v>31</v>
-      </c>
-      <c r="D5" t="s">
-        <v>32</v>
       </c>
       <c r="E5" t="s">
         <v>25</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G5">
         <v>3000</v>
       </c>
       <c r="H5">
-        <v>35</v>
+        <v>39.74</v>
       </c>
       <c r="I5">
-        <v>105000</v>
+        <v>119220</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -2603,25 +2604,25 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
         <v>25</v>
       </c>
       <c r="F6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G6">
         <v>3000</v>
       </c>
       <c r="H6">
-        <v>44.88</v>
+        <v>47.6</v>
       </c>
       <c r="I6">
-        <v>134640</v>
+        <v>142800</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -2635,16 +2636,16 @@
         <v>25</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G7">
         <v>3000</v>
       </c>
       <c r="H7">
-        <v>37.119999999999997</v>
+        <v>36.15</v>
       </c>
       <c r="I7">
-        <v>111360</v>
+        <v>108450</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -2655,25 +2656,22 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E8" t="s">
         <v>25</v>
       </c>
       <c r="F8">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G8">
         <v>3000</v>
       </c>
       <c r="H8">
-        <v>40.29</v>
+        <v>40</v>
       </c>
       <c r="I8">
-        <v>120870</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -2684,25 +2682,25 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
         <v>25</v>
       </c>
       <c r="F9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G9">
         <v>3000</v>
       </c>
       <c r="H9">
-        <v>37</v>
+        <v>36.950000000000003</v>
       </c>
       <c r="I9">
-        <v>111000</v>
+        <v>110850</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -2712,20 +2710,26 @@
       <c r="B10" t="s">
         <v>8</v>
       </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" t="s">
+        <v>35</v>
+      </c>
       <c r="E10" t="s">
         <v>25</v>
       </c>
       <c r="F10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G10">
         <v>3000</v>
       </c>
       <c r="H10">
-        <v>38</v>
+        <v>42.84</v>
       </c>
       <c r="I10">
-        <v>114000</v>
+        <v>128520</v>
       </c>
     </row>
   </sheetData>
@@ -2749,25 +2753,25 @@
     <col min="9" max="9" width="31.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="38.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="14" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13" bestFit="1" customWidth="1"/>
     <col min="20" max="21" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="23.42578125" bestFit="1" customWidth="1"/>
     <col min="34" max="35" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -2785,7 +2789,7 @@
     <col min="51" max="51" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="27.5703125" bestFit="1" customWidth="1"/>
     <col min="55" max="56" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="57" max="57" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="58" max="58" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -2797,7 +2801,7 @@
     <col min="65" max="65" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="66" max="66" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="67" max="67" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="69" max="70" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="71" max="71" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="72" max="72" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -2845,19 +2849,19 @@
         <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>10</v>
@@ -3075,168 +3079,168 @@
         <v>25</v>
       </c>
       <c r="M3">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="N3">
         <v>3000</v>
       </c>
       <c r="O3">
-        <v>69.5</v>
+        <v>40</v>
       </c>
       <c r="P3">
-        <v>208500</v>
+        <v>120000</v>
       </c>
       <c r="S3" t="s">
         <v>25</v>
       </c>
       <c r="T3">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="U3">
         <v>3000</v>
       </c>
       <c r="V3">
-        <v>36.36</v>
+        <v>56</v>
       </c>
       <c r="W3">
-        <v>109080</v>
+        <v>168000</v>
       </c>
       <c r="Z3" t="s">
         <v>25</v>
       </c>
       <c r="AA3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AB3">
         <v>3000</v>
       </c>
       <c r="AC3">
-        <v>40.5</v>
+        <v>40.049999999999997</v>
       </c>
       <c r="AD3">
-        <v>121500</v>
+        <v>120150</v>
       </c>
       <c r="AG3" t="s">
         <v>25</v>
       </c>
       <c r="AH3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AI3">
         <v>3000</v>
       </c>
       <c r="AJ3">
-        <v>35</v>
+        <v>39.74</v>
       </c>
       <c r="AK3">
-        <v>105000</v>
+        <v>119220</v>
       </c>
       <c r="AN3" t="s">
         <v>25</v>
       </c>
       <c r="AO3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP3">
         <v>3000</v>
       </c>
       <c r="AQ3">
-        <v>44.88</v>
+        <v>47.6</v>
       </c>
       <c r="AR3">
-        <v>134640</v>
+        <v>142800</v>
       </c>
       <c r="AU3" t="s">
         <v>25</v>
       </c>
       <c r="AV3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AW3">
         <v>3000</v>
       </c>
       <c r="AX3">
-        <v>37.119999999999997</v>
+        <v>36.15</v>
       </c>
       <c r="AY3">
-        <v>111360</v>
+        <v>108450</v>
       </c>
       <c r="BB3" t="s">
         <v>25</v>
       </c>
       <c r="BC3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BD3">
         <v>3000</v>
       </c>
       <c r="BE3">
-        <v>40.29</v>
+        <v>40</v>
       </c>
       <c r="BF3">
-        <v>120870</v>
+        <v>120000</v>
       </c>
       <c r="BI3" t="s">
         <v>25</v>
       </c>
       <c r="BJ3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BK3">
         <v>3000</v>
       </c>
       <c r="BL3">
-        <v>37</v>
+        <v>36.950000000000003</v>
       </c>
       <c r="BM3">
-        <v>111000</v>
+        <v>110850</v>
       </c>
       <c r="BP3" t="s">
         <v>25</v>
       </c>
       <c r="BQ3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BR3">
         <v>3000</v>
       </c>
       <c r="BS3">
-        <v>38</v>
+        <v>42.84</v>
       </c>
       <c r="BT3">
-        <v>114000</v>
+        <v>128520</v>
       </c>
     </row>
     <row r="5" spans="1:74" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P5">
-        <v>208500</v>
+        <v>120000</v>
       </c>
       <c r="W5">
-        <v>109080</v>
+        <v>168000</v>
       </c>
       <c r="AD5">
-        <v>121500</v>
+        <v>120150</v>
       </c>
       <c r="AK5">
-        <v>105000</v>
+        <v>119220</v>
       </c>
       <c r="AR5">
-        <v>134640</v>
+        <v>142800</v>
       </c>
       <c r="AY5">
-        <v>111360</v>
+        <v>108450</v>
       </c>
       <c r="BF5">
-        <v>120870</v>
+        <v>120000</v>
       </c>
       <c r="BM5">
-        <v>111000</v>
+        <v>110850</v>
       </c>
       <c r="BT5">
-        <v>114000</v>
+        <v>128520</v>
       </c>
     </row>
   </sheetData>
@@ -3249,27 +3253,27 @@
   <dimension ref="A2:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+    </row>
+    <row r="3" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-    </row>
-    <row r="3" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3277,7 +3281,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3285,7 +3289,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3293,23 +3297,23 @@
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3317,7 +3321,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3325,7 +3329,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3333,7 +3337,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3342,6 +3346,9 @@
       </c>
       <c r="B12" s="2" t="s">
         <v>47</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rework bid dashboard around base-year vs comparison-year analysis
</commit_message>
<xml_diff>
--- a/support/2026.xlsx
+++ b/support/2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Purchasing\1 All solicitations in progress\B U-CHANNEL SIGN POSTS\TABS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rcoc-my.sharepoint.com/personal/abates_rcoc_org/Documents/Documents/GitHub/bidAnalysis/support/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09ED5BA9-48C3-47D2-B0AA-9A4973C1BA38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{09ED5BA9-48C3-47D2-B0AA-9A4973C1BA38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0CDB3E7-B18E-4797-9317-578EC73247BD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Price Analysis" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="92">
   <si>
     <t>CANUCK POWER INC</t>
   </si>
@@ -441,6 +441,9 @@
   <si>
     <t>14-18 weeks</t>
   </si>
+  <si>
+    <t>Item Number</t>
+  </si>
 </sst>
 </file>
 
@@ -450,7 +453,7 @@
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -528,6 +531,14 @@
     </font>
     <font>
       <i/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Aptos Narrow"/>
@@ -695,7 +706,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -721,23 +732,26 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -748,31 +762,29 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="6" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1174,239 +1186,239 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="13" t="s">
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="13" t="s">
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="14"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="28"/>
     </row>
     <row r="6" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="19" t="s">
+      <c r="B6" s="13"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="19" t="s">
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="19" t="s">
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="M6" s="20"/>
-      <c r="N6" s="20"/>
-      <c r="O6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="22"/>
     </row>
     <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="20"/>
-      <c r="J7" s="20"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="20"/>
-      <c r="N7" s="20"/>
-      <c r="O7" s="21"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="20"/>
+      <c r="M7" s="21"/>
+      <c r="N7" s="21"/>
+      <c r="O7" s="22"/>
     </row>
     <row r="8" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="19" t="s">
+      <c r="B8" s="13"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="19" t="s">
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="20"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="19" t="s">
+      <c r="I8" s="21"/>
+      <c r="J8" s="21"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="M8" s="20"/>
-      <c r="N8" s="20"/>
-      <c r="O8" s="21"/>
+      <c r="M8" s="21"/>
+      <c r="N8" s="21"/>
+      <c r="O8" s="22"/>
     </row>
     <row r="9" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="19" t="s">
+      <c r="B9" s="13"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="19" t="s">
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="I9" s="20"/>
-      <c r="J9" s="20"/>
-      <c r="K9" s="21"/>
-      <c r="L9" s="19">
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="20">
         <v>500</v>
       </c>
-      <c r="M9" s="20"/>
-      <c r="N9" s="20"/>
-      <c r="O9" s="21"/>
+      <c r="M9" s="21"/>
+      <c r="N9" s="21"/>
+      <c r="O9" s="22"/>
     </row>
     <row r="10" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="19">
+      <c r="B10" s="13"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="20">
         <v>45</v>
       </c>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="19" t="s">
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="19">
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="20">
         <v>120</v>
       </c>
-      <c r="M10" s="20"/>
-      <c r="N10" s="20"/>
-      <c r="O10" s="21"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="21"/>
+      <c r="O10" s="22"/>
     </row>
     <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="19">
+      <c r="B11" s="13"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="20">
         <v>50</v>
       </c>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="19">
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="20">
         <v>50</v>
       </c>
-      <c r="I11" s="20"/>
-      <c r="J11" s="20"/>
-      <c r="K11" s="21"/>
-      <c r="L11" s="19">
+      <c r="I11" s="21"/>
+      <c r="J11" s="21"/>
+      <c r="K11" s="22"/>
+      <c r="L11" s="20">
         <v>50</v>
       </c>
-      <c r="M11" s="20"/>
-      <c r="N11" s="20"/>
-      <c r="O11" s="21"/>
+      <c r="M11" s="21"/>
+      <c r="N11" s="21"/>
+      <c r="O11" s="22"/>
     </row>
     <row r="12" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="19" t="s">
+      <c r="B12" s="13"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="19" t="s">
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="21"/>
-      <c r="L12" s="19" t="s">
+      <c r="I12" s="21"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="22"/>
+      <c r="L12" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M12" s="20"/>
-      <c r="N12" s="20"/>
-      <c r="O12" s="21"/>
+      <c r="M12" s="21"/>
+      <c r="N12" s="21"/>
+      <c r="O12" s="22"/>
     </row>
     <row r="13" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="20"/>
-      <c r="J13" s="20"/>
-      <c r="K13" s="21"/>
-      <c r="L13" s="19" t="s">
+      <c r="B13" s="13"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="21"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="M13" s="20"/>
-      <c r="N13" s="20"/>
-      <c r="O13" s="21"/>
+      <c r="M13" s="21"/>
+      <c r="N13" s="21"/>
+      <c r="O13" s="22"/>
     </row>
     <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="19" t="s">
+      <c r="B14" s="15"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="19" t="s">
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
-      <c r="K14" s="21"/>
-      <c r="L14" s="19" t="s">
+      <c r="I14" s="21"/>
+      <c r="J14" s="21"/>
+      <c r="K14" s="22"/>
+      <c r="L14" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M14" s="20"/>
-      <c r="N14" s="20"/>
-      <c r="O14" s="21"/>
+      <c r="M14" s="21"/>
+      <c r="N14" s="21"/>
+      <c r="O14" s="22"/>
     </row>
     <row r="15" spans="1:15" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
@@ -1499,265 +1511,265 @@
       </c>
     </row>
     <row r="17" spans="1:15" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="24"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="19"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="17">
+      <c r="F17" s="25">
         <v>108450</v>
       </c>
-      <c r="G17" s="18"/>
+      <c r="G17" s="26"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="17">
+      <c r="J17" s="25">
         <v>110850</v>
       </c>
-      <c r="K17" s="18"/>
+      <c r="K17" s="26"/>
       <c r="L17" s="12"/>
       <c r="M17" s="12"/>
-      <c r="N17" s="17">
+      <c r="N17" s="25">
         <v>119220</v>
       </c>
-      <c r="O17" s="18"/>
+      <c r="O17" s="26"/>
     </row>
     <row r="18" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="1:15" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="13" t="s">
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="13" t="s">
+      <c r="I19" s="28"/>
+      <c r="J19" s="28"/>
+      <c r="K19" s="28"/>
+      <c r="L19" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="M19" s="14"/>
-      <c r="N19" s="14"/>
-      <c r="O19" s="14"/>
+      <c r="M19" s="28"/>
+      <c r="N19" s="28"/>
+      <c r="O19" s="28"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
+      <c r="A20" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="15"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="19" t="s">
+      <c r="B20" s="13"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="19" t="s">
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="I20" s="20"/>
-      <c r="J20" s="20"/>
-      <c r="K20" s="21"/>
-      <c r="L20" s="19" t="s">
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="M20" s="20"/>
-      <c r="N20" s="20"/>
-      <c r="O20" s="21"/>
+      <c r="M20" s="21"/>
+      <c r="N20" s="21"/>
+      <c r="O20" s="22"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="19" t="s">
+      <c r="B21" s="13"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="I21" s="20"/>
-      <c r="J21" s="20"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="19"/>
-      <c r="M21" s="20"/>
-      <c r="N21" s="20"/>
-      <c r="O21" s="21"/>
+      <c r="I21" s="21"/>
+      <c r="J21" s="21"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="20"/>
+      <c r="M21" s="21"/>
+      <c r="N21" s="21"/>
+      <c r="O21" s="22"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="19" t="s">
+      <c r="B22" s="13"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="19" t="s">
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="I22" s="20"/>
-      <c r="J22" s="20"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="19" t="s">
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="M22" s="20"/>
-      <c r="N22" s="20"/>
-      <c r="O22" s="21"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
+      <c r="O22" s="22"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="B23" s="15"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="27">
+      <c r="B23" s="13"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="24">
         <v>30000</v>
       </c>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="19" t="s">
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="21"/>
-      <c r="L23" s="19" t="s">
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="M23" s="20"/>
-      <c r="N23" s="20"/>
-      <c r="O23" s="21"/>
+      <c r="M23" s="21"/>
+      <c r="N23" s="21"/>
+      <c r="O23" s="22"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B24" s="15"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="19" t="s">
+      <c r="B24" s="13"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="19" t="s">
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="I24" s="20"/>
-      <c r="J24" s="20"/>
-      <c r="K24" s="21"/>
-      <c r="L24" s="19" t="s">
+      <c r="I24" s="21"/>
+      <c r="J24" s="21"/>
+      <c r="K24" s="22"/>
+      <c r="L24" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="M24" s="20"/>
-      <c r="N24" s="20"/>
-      <c r="O24" s="21"/>
+      <c r="M24" s="21"/>
+      <c r="N24" s="21"/>
+      <c r="O24" s="22"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="19" t="s">
+      <c r="B25" s="13"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="19" t="s">
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="I25" s="20"/>
-      <c r="J25" s="20"/>
-      <c r="K25" s="21"/>
-      <c r="L25" s="19" t="s">
+      <c r="I25" s="21"/>
+      <c r="J25" s="21"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="M25" s="20"/>
-      <c r="N25" s="20"/>
-      <c r="O25" s="21"/>
+      <c r="M25" s="21"/>
+      <c r="N25" s="21"/>
+      <c r="O25" s="22"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
+      <c r="A26" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="15"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="19" t="s">
+      <c r="B26" s="13"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="19" t="s">
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="I26" s="20"/>
-      <c r="J26" s="20"/>
-      <c r="K26" s="21"/>
-      <c r="L26" s="19"/>
-      <c r="M26" s="20"/>
-      <c r="N26" s="20"/>
-      <c r="O26" s="21"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="21"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="20"/>
+      <c r="M26" s="21"/>
+      <c r="N26" s="21"/>
+      <c r="O26" s="22"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="15" t="s">
+      <c r="A27" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="B27" s="15"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="19" t="s">
+      <c r="B27" s="13"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="I27" s="20"/>
-      <c r="J27" s="20"/>
-      <c r="K27" s="21"/>
-      <c r="L27" s="19"/>
-      <c r="M27" s="20"/>
-      <c r="N27" s="20"/>
-      <c r="O27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="20"/>
+      <c r="M27" s="21"/>
+      <c r="N27" s="21"/>
+      <c r="O27" s="22"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="19" t="s">
+      <c r="B28" s="15"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="19" t="s">
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="I28" s="20"/>
-      <c r="J28" s="20"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="19" t="s">
+      <c r="I28" s="21"/>
+      <c r="J28" s="21"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M28" s="20"/>
-      <c r="N28" s="20"/>
-      <c r="O28" s="21"/>
+      <c r="M28" s="21"/>
+      <c r="N28" s="21"/>
+      <c r="O28" s="22"/>
     </row>
     <row r="29" spans="1:15" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
@@ -1850,258 +1862,258 @@
       </c>
     </row>
     <row r="31" spans="1:15" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="22" t="s">
+      <c r="A31" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="23"/>
-      <c r="C31" s="24"/>
+      <c r="B31" s="18"/>
+      <c r="C31" s="19"/>
       <c r="D31" s="12"/>
       <c r="E31" s="12"/>
-      <c r="F31" s="17">
+      <c r="F31" s="25">
         <v>120000</v>
       </c>
-      <c r="G31" s="18"/>
+      <c r="G31" s="26"/>
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
-      <c r="J31" s="17">
+      <c r="J31" s="25">
         <v>120000</v>
       </c>
-      <c r="K31" s="18"/>
+      <c r="K31" s="26"/>
       <c r="L31" s="12"/>
       <c r="M31" s="12"/>
-      <c r="N31" s="17">
+      <c r="N31" s="25">
         <v>120150</v>
       </c>
-      <c r="O31" s="18"/>
+      <c r="O31" s="26"/>
     </row>
     <row r="39" spans="1:15" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D39" s="13" t="s">
+      <c r="D39" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="13" t="s">
+      <c r="E39" s="28"/>
+      <c r="F39" s="28"/>
+      <c r="G39" s="28"/>
+      <c r="H39" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="I39" s="14"/>
-      <c r="J39" s="14"/>
-      <c r="K39" s="14"/>
-      <c r="L39" s="13" t="s">
+      <c r="I39" s="28"/>
+      <c r="J39" s="28"/>
+      <c r="K39" s="28"/>
+      <c r="L39" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="M39" s="14"/>
-      <c r="N39" s="14"/>
-      <c r="O39" s="14"/>
+      <c r="M39" s="28"/>
+      <c r="N39" s="28"/>
+      <c r="O39" s="28"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A40" s="15" t="s">
+      <c r="A40" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B40" s="15"/>
-      <c r="C40" s="16"/>
-      <c r="D40" s="19" t="s">
+      <c r="B40" s="13"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="21"/>
-      <c r="H40" s="19" t="s">
+      <c r="E40" s="21"/>
+      <c r="F40" s="21"/>
+      <c r="G40" s="22"/>
+      <c r="H40" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="I40" s="20"/>
-      <c r="J40" s="20"/>
-      <c r="K40" s="21"/>
-      <c r="L40" s="19" t="s">
+      <c r="I40" s="21"/>
+      <c r="J40" s="21"/>
+      <c r="K40" s="22"/>
+      <c r="L40" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="M40" s="20"/>
-      <c r="N40" s="20"/>
-      <c r="O40" s="21"/>
+      <c r="M40" s="21"/>
+      <c r="N40" s="21"/>
+      <c r="O40" s="22"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="15" t="s">
+      <c r="A41" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B41" s="15"/>
-      <c r="C41" s="16"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="20"/>
-      <c r="F41" s="20"/>
-      <c r="G41" s="21"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="20"/>
-      <c r="J41" s="20"/>
-      <c r="K41" s="21"/>
-      <c r="L41" s="19"/>
-      <c r="M41" s="20"/>
-      <c r="N41" s="20"/>
-      <c r="O41" s="21"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="20"/>
+      <c r="I41" s="21"/>
+      <c r="J41" s="21"/>
+      <c r="K41" s="22"/>
+      <c r="L41" s="20"/>
+      <c r="M41" s="21"/>
+      <c r="N41" s="21"/>
+      <c r="O41" s="22"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A42" s="15" t="s">
+      <c r="A42" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B42" s="15"/>
-      <c r="C42" s="16"/>
-      <c r="D42" s="28">
+      <c r="B42" s="13"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="23">
         <v>46387</v>
       </c>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="21"/>
-      <c r="H42" s="19" t="s">
+      <c r="E42" s="21"/>
+      <c r="F42" s="21"/>
+      <c r="G42" s="22"/>
+      <c r="H42" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="I42" s="20"/>
-      <c r="J42" s="20"/>
-      <c r="K42" s="21"/>
-      <c r="L42" s="19" t="s">
+      <c r="I42" s="21"/>
+      <c r="J42" s="21"/>
+      <c r="K42" s="22"/>
+      <c r="L42" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="M42" s="20"/>
-      <c r="N42" s="20"/>
-      <c r="O42" s="21"/>
+      <c r="M42" s="21"/>
+      <c r="N42" s="21"/>
+      <c r="O42" s="22"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="15" t="s">
+      <c r="A43" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="B43" s="15"/>
-      <c r="C43" s="16"/>
-      <c r="D43" s="19" t="s">
+      <c r="B43" s="13"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="E43" s="20"/>
-      <c r="F43" s="20"/>
-      <c r="G43" s="21"/>
-      <c r="H43" s="19"/>
-      <c r="I43" s="20"/>
-      <c r="J43" s="20"/>
-      <c r="K43" s="21"/>
-      <c r="L43" s="19" t="s">
+      <c r="E43" s="21"/>
+      <c r="F43" s="21"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="20"/>
+      <c r="I43" s="21"/>
+      <c r="J43" s="21"/>
+      <c r="K43" s="22"/>
+      <c r="L43" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="M43" s="20"/>
-      <c r="N43" s="20"/>
-      <c r="O43" s="21"/>
+      <c r="M43" s="21"/>
+      <c r="N43" s="21"/>
+      <c r="O43" s="22"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44" s="15" t="s">
+      <c r="A44" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B44" s="15"/>
-      <c r="C44" s="16"/>
-      <c r="D44" s="19" t="s">
+      <c r="B44" s="13"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="E44" s="20"/>
-      <c r="F44" s="20"/>
-      <c r="G44" s="21"/>
-      <c r="H44" s="19" t="s">
+      <c r="E44" s="21"/>
+      <c r="F44" s="21"/>
+      <c r="G44" s="22"/>
+      <c r="H44" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="I44" s="20"/>
-      <c r="J44" s="20"/>
-      <c r="K44" s="21"/>
-      <c r="L44" s="19" t="s">
+      <c r="I44" s="21"/>
+      <c r="J44" s="21"/>
+      <c r="K44" s="22"/>
+      <c r="L44" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="M44" s="20"/>
-      <c r="N44" s="20"/>
-      <c r="O44" s="21"/>
+      <c r="M44" s="21"/>
+      <c r="N44" s="21"/>
+      <c r="O44" s="22"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45" s="15" t="s">
+      <c r="A45" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B45" s="15"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="19">
+      <c r="B45" s="13"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="20">
         <v>50</v>
       </c>
-      <c r="E45" s="20"/>
-      <c r="F45" s="20"/>
-      <c r="G45" s="21"/>
-      <c r="H45" s="19" t="s">
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="22"/>
+      <c r="H45" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="I45" s="20"/>
-      <c r="J45" s="20"/>
-      <c r="K45" s="21"/>
-      <c r="L45" s="19"/>
-      <c r="M45" s="20"/>
-      <c r="N45" s="20"/>
-      <c r="O45" s="21"/>
+      <c r="I45" s="21"/>
+      <c r="J45" s="21"/>
+      <c r="K45" s="22"/>
+      <c r="L45" s="20"/>
+      <c r="M45" s="21"/>
+      <c r="N45" s="21"/>
+      <c r="O45" s="22"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A46" s="15" t="s">
+      <c r="A46" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B46" s="15"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="19" t="s">
+      <c r="B46" s="13"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="E46" s="20"/>
-      <c r="F46" s="20"/>
-      <c r="G46" s="21"/>
-      <c r="H46" s="19" t="s">
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="I46" s="20"/>
-      <c r="J46" s="20"/>
-      <c r="K46" s="21"/>
-      <c r="L46" s="19" t="s">
+      <c r="I46" s="21"/>
+      <c r="J46" s="21"/>
+      <c r="K46" s="22"/>
+      <c r="L46" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="M46" s="20"/>
-      <c r="N46" s="20"/>
-      <c r="O46" s="21"/>
+      <c r="M46" s="21"/>
+      <c r="N46" s="21"/>
+      <c r="O46" s="22"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A47" s="15" t="s">
+      <c r="A47" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="B47" s="15"/>
-      <c r="C47" s="16"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="20"/>
-      <c r="F47" s="20"/>
-      <c r="G47" s="21"/>
-      <c r="H47" s="19"/>
-      <c r="I47" s="20"/>
-      <c r="J47" s="20"/>
-      <c r="K47" s="21"/>
-      <c r="L47" s="19"/>
-      <c r="M47" s="20"/>
-      <c r="N47" s="20"/>
-      <c r="O47" s="21"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="22"/>
+      <c r="H47" s="20"/>
+      <c r="I47" s="21"/>
+      <c r="J47" s="21"/>
+      <c r="K47" s="22"/>
+      <c r="L47" s="20"/>
+      <c r="M47" s="21"/>
+      <c r="N47" s="21"/>
+      <c r="O47" s="22"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="25" t="s">
+      <c r="A48" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="B48" s="25"/>
-      <c r="C48" s="26"/>
-      <c r="D48" s="19" t="s">
+      <c r="B48" s="15"/>
+      <c r="C48" s="16"/>
+      <c r="D48" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="21"/>
-      <c r="H48" s="19" t="s">
+      <c r="E48" s="21"/>
+      <c r="F48" s="21"/>
+      <c r="G48" s="22"/>
+      <c r="H48" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="I48" s="20"/>
-      <c r="J48" s="20"/>
-      <c r="K48" s="21"/>
-      <c r="L48" s="19" t="s">
+      <c r="I48" s="21"/>
+      <c r="J48" s="21"/>
+      <c r="K48" s="22"/>
+      <c r="L48" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M48" s="20"/>
-      <c r="N48" s="20"/>
-      <c r="O48" s="21"/>
+      <c r="M48" s="21"/>
+      <c r="N48" s="21"/>
+      <c r="O48" s="22"/>
     </row>
     <row r="49" spans="1:15" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
@@ -2198,52 +2210,117 @@
       </c>
     </row>
     <row r="51" spans="1:15" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="22" t="s">
+      <c r="A51" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B51" s="23"/>
-      <c r="C51" s="24"/>
+      <c r="B51" s="18"/>
+      <c r="C51" s="19"/>
       <c r="D51" s="12"/>
       <c r="E51" s="12"/>
-      <c r="F51" s="17">
+      <c r="F51" s="25">
         <v>128520</v>
       </c>
-      <c r="G51" s="18"/>
+      <c r="G51" s="26"/>
       <c r="H51" s="12"/>
       <c r="I51" s="12"/>
-      <c r="J51" s="17">
+      <c r="J51" s="25">
         <v>142800</v>
       </c>
-      <c r="K51" s="18"/>
+      <c r="K51" s="26"/>
       <c r="L51" s="12"/>
       <c r="M51" s="12"/>
-      <c r="N51" s="17">
+      <c r="N51" s="25">
         <v>168000</v>
       </c>
-      <c r="O51" s="18"/>
+      <c r="O51" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="129">
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="L5:O5"/>
+    <mergeCell ref="H5:K5"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="L7:O7"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="L10:O10"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="J51:K51"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="L45:O45"/>
+    <mergeCell ref="L46:O46"/>
+    <mergeCell ref="L48:O48"/>
+    <mergeCell ref="L47:O47"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="N31:O31"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="L39:O39"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="D28:G28"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="D45:G45"/>
+    <mergeCell ref="D46:G46"/>
+    <mergeCell ref="D48:G48"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="H8:K8"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="L11:O11"/>
+    <mergeCell ref="L12:O12"/>
+    <mergeCell ref="L14:O14"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="L44:O44"/>
+    <mergeCell ref="H40:K40"/>
+    <mergeCell ref="H41:K41"/>
+    <mergeCell ref="H42:K42"/>
+    <mergeCell ref="H43:K43"/>
+    <mergeCell ref="H44:K44"/>
+    <mergeCell ref="D39:G39"/>
+    <mergeCell ref="L19:O19"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="H45:K45"/>
+    <mergeCell ref="H46:K46"/>
+    <mergeCell ref="H48:K48"/>
+    <mergeCell ref="D47:G47"/>
+    <mergeCell ref="H47:K47"/>
+    <mergeCell ref="D40:G40"/>
+    <mergeCell ref="D41:G41"/>
+    <mergeCell ref="D42:G42"/>
+    <mergeCell ref="D43:G43"/>
+    <mergeCell ref="D44:G44"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="D13:G13"/>
     <mergeCell ref="H13:K13"/>
@@ -2268,91 +2345,26 @@
     <mergeCell ref="L27:O27"/>
     <mergeCell ref="H20:K20"/>
     <mergeCell ref="H21:K21"/>
-    <mergeCell ref="H45:K45"/>
-    <mergeCell ref="H46:K46"/>
-    <mergeCell ref="H48:K48"/>
-    <mergeCell ref="D47:G47"/>
-    <mergeCell ref="H47:K47"/>
-    <mergeCell ref="D40:G40"/>
-    <mergeCell ref="D41:G41"/>
-    <mergeCell ref="D42:G42"/>
-    <mergeCell ref="D43:G43"/>
-    <mergeCell ref="D44:G44"/>
-    <mergeCell ref="L11:O11"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="L14:O14"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="L44:O44"/>
-    <mergeCell ref="H40:K40"/>
-    <mergeCell ref="H41:K41"/>
-    <mergeCell ref="H42:K42"/>
-    <mergeCell ref="H43:K43"/>
-    <mergeCell ref="H44:K44"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="H8:K8"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="D6:G6"/>
-    <mergeCell ref="D7:G7"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="J51:K51"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="L45:O45"/>
-    <mergeCell ref="L46:O46"/>
-    <mergeCell ref="L48:O48"/>
-    <mergeCell ref="L47:O47"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="L39:O39"/>
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="D28:G28"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="D45:G45"/>
-    <mergeCell ref="D46:G46"/>
-    <mergeCell ref="D48:G48"/>
-    <mergeCell ref="D39:G39"/>
-    <mergeCell ref="L19:O19"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="L5:O5"/>
-    <mergeCell ref="H5:K5"/>
-    <mergeCell ref="D5:G5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="L7:O7"/>
-    <mergeCell ref="L8:O8"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="L10:O10"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A44:C44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="3" scale="90" fitToWidth="0" orientation="landscape" verticalDpi="0" r:id="rId1"/>
@@ -2361,68 +2373,74 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C2" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
         <v>23</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>22</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>24</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>3000</v>
       </c>
     </row>

</xml_diff>